<commit_message>
Group B: female ORB port leg (leg_ORBPORT + ORBMOUTH revolved cut) and SPECs 6815 / 6832 / 6835 from the Brennan catalog: 14 configurations; dofcheck / allcfg extended; OCP closed loop 0 off (ports = Brennan STEP ports)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6815.xlsx
+++ b/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6815.xlsx
@@ -413,43 +413,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>OMi 6815 - Design Table SKELETON (no dimensional source) | OMi catalog 6 SKUs | ALL MISSING | GENERATED 2026-09-23</t>
+          <t>OMi 6815 - review table | Brennan TFA catalog TFA-p045-t01 + Brennan CAD records (group B 2026-10-21); port drill = Air-Way per-size (A11) | was a skeleton</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
+          <t>M8@DRIVE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>M6@DRIVE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>D1@BORE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CHEX@HEX</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y@HEX</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PD@BORE</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>THDMAJ_B1@DRIVE</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>$PRP@DimSource</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>$PRP@PartNo</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>$PRP@DataStatus</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>$PRP@AxialSource</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>$PRP@ScopeAction</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>$PRP@OMiSKU</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>$COMMENT</t>
         </is>
@@ -461,32 +501,58 @@
           <t>6815-04-04-NWO-FG</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.5629999999999999</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>6815-04-04-NWO-FG</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAT 2026-10-21: M8@DRIVE, M6@DRIVE, D1@BORE, CHEX@HEX, Y@HEX] Brennan TFA catalog TFA-p045-t01 (CAD record agrees within the print rounding); port drill PD@BORE = Air-Way per-size (A11) [user 2026-10-18 "Brennan = yes"; 2026-10-21 CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>6815-04-04-NWO-FG</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
         </is>
@@ -498,32 +564,58 @@
           <t>6815-06-06-NWO-FG</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.297</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>6815-06-06-NWO-FG</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAT 2026-10-21: M8@DRIVE, M6@DRIVE, D1@BORE, CHEX@HEX, Y@HEX] Brennan TFA catalog TFA-p045-t01 (CAD record agrees within the print rounding); port drill PD@BORE = Air-Way per-size (A11) [user 2026-10-18 "Brennan = yes"; 2026-10-21 CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>6815-06-06-NWO-FG</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
         </is>
@@ -535,32 +627,58 @@
           <t>6815-08-08-NWO-FG</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.391</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.062</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>6815-08-08-NWO-FG</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAT 2026-10-21: M8@DRIVE, M6@DRIVE, D1@BORE, CHEX@HEX, Y@HEX] Brennan TFA catalog TFA-p045-t01 (CAD record agrees within the print rounding); port drill PD@BORE = Air-Way per-size (A11) [user 2026-10-18 "Brennan = yes"; 2026-10-21 CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>6815-08-08-NWO-FG</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
         </is>
@@ -572,32 +690,58 @@
           <t>6815-10-10-NWO-FG</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.062</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>6815-10-10-NWO-FG</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAT 2026-10-21: M8@DRIVE, M6@DRIVE, D1@BORE, CHEX@HEX, Y@HEX] Brennan TFA catalog TFA-p045-t01 (CAD record agrees within the print rounding); port drill PD@BORE = Air-Way per-size (A11) [user 2026-10-18 "Brennan = yes"; 2026-10-21 CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>6815-10-10-NWO-FG</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
         </is>
@@ -609,32 +753,58 @@
           <t>6815-12-12-NWO-FG</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.609</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.0625</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>6815-12-12-NWO-FG</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAT 2026-10-21: M8@DRIVE, M6@DRIVE, D1@BORE, CHEX@HEX, Y@HEX] Brennan TFA catalog TFA-p045-t01 (CAD record agrees within the print rounding); port drill PD@BORE = Air-Way per-size (A11) [user 2026-10-18 "Brennan = yes"; 2026-10-21 CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>6815-12-12-NWO-FG</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
         </is>
@@ -646,32 +816,58 @@
           <t>6815-16-16-NWO-FG</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.3125</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>6815-16-16-NWO-FG</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAT 2026-10-21: M8@DRIVE, M6@DRIVE, D1@BORE, CHEX@HEX, Y@HEX] Brennan TFA catalog TFA-p045-t01 (CAD record agrees within the print rounding); port drill PD@BORE = Air-Way per-size (A11) [user 2026-10-18 "Brennan = yes"; 2026-10-21 CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>6815-16-16-NWO-FG</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
         </is>

</xml_diff>